<commit_message>
feat: Refactor imports to streamline module structure and add utility functions for data processing
</commit_message>
<xml_diff>
--- a/dataset_statistics.xlsx
+++ b/dataset_statistics.xlsx
@@ -477,16 +477,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.001151069039593282</v>
+        <v>9.467231464441011e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>-1.19919152395404</v>
+        <v>-1.199896671404731</v>
       </c>
       <c r="D2" t="n">
-        <v>101</v>
+        <v>389</v>
       </c>
       <c r="E2" t="n">
-        <v>1980.19801980198</v>
+        <v>514.1388174807198</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -495,7 +495,7 @@
         <v>200000</v>
       </c>
       <c r="H2" t="n">
-        <v>1000000</v>
+        <v>60000000</v>
       </c>
     </row>
     <row r="3">
@@ -505,16 +505,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.001819595196333088</v>
+        <v>0.000402335634019715</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.07773034599960971</v>
+        <v>-0.07938209342390801</v>
       </c>
       <c r="D3" t="n">
-        <v>221</v>
+        <v>869</v>
       </c>
       <c r="E3" t="n">
-        <v>904.9773755656108</v>
+        <v>230.1495972382048</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -523,7 +523,7 @@
         <v>200000</v>
       </c>
       <c r="H3" t="n">
-        <v>1000000</v>
+        <v>60000000</v>
       </c>
     </row>
     <row r="4">
@@ -533,10 +533,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>322.7127753034191</v>
+        <v>302.0200487576828</v>
       </c>
       <c r="C4" t="n">
-        <v>146646.6829839263</v>
+        <v>107173.5809963281</v>
       </c>
       <c r="D4" t="n">
         <v>2000</v>
@@ -551,7 +551,7 @@
         <v>200000</v>
       </c>
       <c r="H4" t="n">
-        <v>1000000</v>
+        <v>60000000</v>
       </c>
     </row>
     <row r="5">
@@ -561,25 +561,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.03617830564667604</v>
+        <v>0.6865509635457695</v>
       </c>
       <c r="C5" t="n">
-        <v>-1.47207122738883</v>
+        <v>-1.314084349633445</v>
       </c>
       <c r="D5" t="n">
-        <v>71</v>
+        <v>228</v>
       </c>
       <c r="E5" t="n">
-        <v>1996.549295774648</v>
+        <v>734.1447368421053</v>
       </c>
       <c r="F5" t="n">
-        <v>19762</v>
+        <v>17540</v>
       </c>
       <c r="G5" t="n">
-        <v>161517</v>
+        <v>184925</v>
       </c>
       <c r="H5" t="n">
-        <v>1000000</v>
+        <v>60000000</v>
       </c>
     </row>
     <row r="6">
@@ -589,16 +589,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.001865259250622435</v>
+        <v>4.931911190539385e-05</v>
       </c>
       <c r="C6" t="n">
-        <v>-1.199400424667698</v>
+        <v>-1.19993843329877</v>
       </c>
       <c r="D6" t="n">
-        <v>99</v>
+        <v>391</v>
       </c>
       <c r="E6" t="n">
-        <v>202.010101010101</v>
+        <v>51.14833759590793</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -607,7 +607,7 @@
         <v>19999</v>
       </c>
       <c r="H6" t="n">
-        <v>1000000</v>
+        <v>60000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>